<commit_message>
Update vendor marketplaces list with status, comments, and Beeline screenshot
- Restored full 18-entry vendor list with verified status for each platform
- Added Comment column with reasons for each status decision
- Updated nextSource status to Applied after submitting supplier form
- Added Beeline registration screenshot for reference

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pro5.ai/Vendor_Marketplaces_List.xlsx
+++ b/Pro5.ai/Vendor_Marketplaces_List.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,10 +35,20 @@
       <color rgb="00006100"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+    </font>
+    <font>
+      <color rgb="00BF6000"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
       <color rgb="009C0006"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +65,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+        <bgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -82,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -94,6 +116,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -461,15 +492,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,6 +536,16 @@
           <t>Priority</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -533,6 +576,16 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Form submitted on Prosperix. Awaiting response.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -563,6 +616,16 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Selected 'Interested in becoming a listed Beeline staffing supplier' option and submitted.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -593,6 +656,16 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Cannot Apply</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Invite-only platform. Clients must invite vendors — no self-registration available.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -623,6 +696,16 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Submitted 'Become a Supplier' form. Selected: Staff Augmentation, SOW, Offshore/Near Shoring, Direct Sourcing. Awaiting response.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -653,6 +736,16 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>1,200+ vetted vendors. Screens for financial stability &amp; certifications. Not a project board — clients find you.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -675,12 +768,22 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>ExonPro consultants can apply individually</t>
+          <t>Apply through their vetting process</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Individual freelancers only. No option for consulting firms to register as a vendor.</t>
         </is>
       </c>
     </row>
@@ -708,9 +811,19 @@
           <t>Good fit for senior Salesforce/Cloud/AI talent</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Primarily for individual consultants. No clear firm/agency registration option.</t>
         </is>
       </c>
     </row>
@@ -720,17 +833,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Talmix</t>
+          <t>Talmix / High5</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>talmix.com</t>
+          <t>high5hire.com</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>65,000+ expert network for business &amp; consulting talent</t>
+          <t>Expert network, now redirects to High5Hire. MSP/VMS integration platform</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -741,6 +854,16 @@
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to High5Hire. Unclear if consulting firms can register. More of an MSP/VMS integration tool.</t>
         </is>
       </c>
     </row>
@@ -760,17 +883,27 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>IT field service marketplace, 20,000+ technicians</t>
+          <t>IT field service marketplace, 20,000+ technicians. On-site/infrastructure focused</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>More infrastructure/on-site focused</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
+          <t>Register as a service company</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Low</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Focused on field service/on-site technicians, not IT consulting or Salesforce projects.</t>
         </is>
       </c>
     </row>
@@ -780,7 +913,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Upwork Enterprise / Lifted</t>
+          <t>Upwork Enterprise</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -801,6 +934,336 @@
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Decided not to apply on Upwork platforms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>FoundHQ</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>foundhq.com</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce-specific marketplace with 8,000+ consultants</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Join as freelancer</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Individual freelancers only. No option for consulting firms — only 'Join as Freelancer' available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Vendorship</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>vendorship.net</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>US government contracting coaching service. Helps businesses bid on federal/SLED contracts</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Paid coaching service for US govt proposals</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>US government contracts only. Paid coaching service, not a free marketplace. Not relevant for India operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>GlobalTenders</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>globaltenders.com</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Global tenders and RFPs for businesses of all sizes</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Register and browse tenders</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Open to businesses of all sizes. Global reach. Worth exploring for IT/Salesforce tenders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>TendersOnTime</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>tendersontime.com</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Global RFPs &amp; RFQs. Has Consultancy RFP category, supports consulting firms</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Register and browse RFPs</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly supports consulting firms. Has dedicated Consultancy RFP category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>HigherGov</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>highergov.com</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>US government contracts and grants for consultants</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Register and browse opportunities</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>US government contracts only. Not relevant for India-based operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Upwork</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>upwork.com</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>4,000+ Salesforce experts listed, active project postings daily</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Create an agency profile and bid on projects</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Decided not to apply on Upwork platforms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Toptal</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>toptal.com</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Curated Salesforce projects with global clients. Top 3% talent</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Apply through their vetting process</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Will Not Apply</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate entry. Individual freelancers only — no firm registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Guru.com</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>guru.com</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>6,800+ Salesforce consultants. Has Guru Agency &amp; Enterprise options</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Register as a team/agency and bid on projects</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Supports agency/enterprise registration. Companies like Scopic (200+ employees) use it. Good fit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update TechnologyMatch status to Cannot Apply — $10M+ revenue required
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pro5.ai/Vendor_Marketplaces_List.xlsx
+++ b/Pro5.ai/Vendor_Marketplaces_List.xlsx
@@ -728,7 +728,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Register on their platform</t>
+          <t>Register at technologymatch.com. Free tier available. Contact: info@technologymatch.com</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Not Applied</t>
+          <t>Cannot Apply</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>1,200+ vetted vendors. Screens for financial stability &amp; certifications. Not a project board — clients find you.</t>
+          <t>Cannot apply — requires $10M+ annual revenue for vendor registration. No US physical location also required. Freemium tier: Free (1 solution page). Premium: $4,800/yr. Enterprise: Custom. Buyers are CIOs/IT directors at mid-market &amp; Fortune 500. Option: Try direct outreach to info@technologymatch.com to request exception for specialized Salesforce consulting.</t>
         </is>
       </c>
     </row>

</xml_diff>